<commit_message>
Add participant age-group coding to pilot workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFWgZDD2Xx2FsxNt9VUonS
</commit_message>
<xml_diff>
--- a/编码/三级编码_试点5篇.xlsx
+++ b/编码/三级编码_试点5篇.xlsx
@@ -430,25 +430,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="25.2" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="36.9" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="20.7" customWidth="1" min="8" max="8"/>
-    <col width="13.5" customWidth="1" min="9" max="9"/>
-    <col width="22.5" customWidth="1" min="10" max="10"/>
-    <col width="15.3" customWidth="1" min="11" max="11"/>
-    <col width="37.8" customWidth="1" min="12" max="12"/>
-    <col width="13.5" customWidth="1" min="13" max="13"/>
-    <col width="12.6" customWidth="1" min="14" max="14"/>
-    <col width="17.1" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="20.7" customWidth="1" min="9" max="9"/>
+    <col width="13.5" customWidth="1" min="10" max="10"/>
+    <col width="22.5" customWidth="1" min="11" max="11"/>
+    <col width="15.3" customWidth="1" min="12" max="12"/>
+    <col width="37.8" customWidth="1" min="13" max="13"/>
+    <col width="13.5" customWidth="1" min="14" max="14"/>
+    <col width="12.6" customWidth="1" min="15" max="15"/>
+    <col width="17.1" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,60 +475,65 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>涉及被试（年龄段）</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>因变量原文名称</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>操作性定义（原文摘录）</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>出处</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>三级编码（暂定）</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>测量单位</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>互动对象</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>剧本/自发</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>是否画图（可算Tau-U）</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>维持数据</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>泛化数据</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>边界标记</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -552,60 +558,65 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Child 1、2、3（均为学龄期）</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Conversational speech (correct response per line of conversation)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>A response was considered correct if the child said the line of the predetermined conversation or any other contextually appropriate statement consisting of an answer and a question.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>PDF第4页</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>会话轮替（回答并提问）</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>每段会话正确轮次数（0–3）</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>治疗师（成人）；泛化含陌生人、兄弟姐妹、孤独症同伴</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>剧本为主，情境适当的新表达也计正确</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>是（图1–3）</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>有（1、2、3、6、15个月）</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>有（人物、情境、话题）</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -626,60 +637,65 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Child 1、2、3（均为学龄期）</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>Question asking (appropriate questions)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>A question was operationally defined as a contextually appropriate verbalization that was asked with the proper intonation and that began with "is," "may," "what," "when," "where," "how," or "can." Prompted questions ... were not included.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>PDF第5页</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>自发提问</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>1.5小时课后活动中的提问次数</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>自然情境（课后项目中的他人）</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>自发</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>是（图4）</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>原文称为附带测量（ancillary），不是直接训练目标</t>
         </is>
@@ -704,60 +720,65 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Child 1、2、3（均为学龄期）</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>Response variation</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>the number of appropriate novel (never said before in the study) responses that differed from the modeled conversations was recorded.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>PDF第5页</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>（不提取）会话中的新异表达</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>百分比</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>治疗师</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>自发</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>否，只在正文报告各阶段百分比</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>未画逐次数据，无法计算Tau-U</t>
         </is>
@@ -782,60 +803,65 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>John（学龄前期）</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>Target social response: "Give it back, please" (John)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>John was taught to say "Give it back, please" within 5 s of an item being taken from his hands. ... Data on correct unprompted occurrences of the target response ... were expressed as the percentage of trials with a correct response.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>PDF第4页</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>索回物品的请求</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>正确试次百分比</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>同伴（视频阶段）；成人</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>固定句式</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>是（图2）</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>见备注</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>本身即泛化探测</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>可能（以获取物品为目的的请求）</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>视频不是最初的干预：先由成人（非视频）教学，视频阶段用于促进向同伴泛化。视频效应单元应为“同伴探测：视频前（PC、SC阶段）vs 视频阶段”，需你确认这样计算是否与原先一致</t>
         </is>
@@ -860,60 +886,65 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>Emma（学龄前期）、Mike（学龄期）</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Target social response: "my turn" (Emma, Mike)</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Emma and Mike were taught to say "my turn" within 5 s after a 1-min timer sounded indicating that the other person's turn with the toy was finished.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>PDF第4页</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>轮流请求（“轮到我了”）</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>正确试次百分比</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>同伴（视频阶段）；成人</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>固定句式</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>是（图2）</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>见上行</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
@@ -938,60 +969,65 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Staci（学龄期）</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Target social response: "What do you want?" (Staci)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>She was taught to ask "What do you want?" when someone indicated a desire for something and Staci was in possession of more than one play item.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>PDF第4页</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>询问他人需求（主动提供帮助）</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>正确试次百分比</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>同伴（视频阶段）；成人</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>固定句式</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>是（图2）</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>见上行</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
@@ -1016,60 +1052,65 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Lucy、Tim、John、Helen（均为学龄前期）</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>Social initiations with peers (physical + vocal)</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Physical initiation was defined as moving into proximity of a peer or group of peers, resulting in some form of engagement. ... Vocal initiation was defined as either verbal (use of words) or nonverbal (vocalization including laughing, crying, and utterances to gain attention).</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>PDF第5页</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>同伴社交发起（肢体接近式+发声/言语式，合并）</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>15分钟操场观察中的次数</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>同伴（自然情境：操场）</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>自发</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>是（图1，只画合并总数）</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>肢体发起与发声发起只在正文按比例描述，图中不分开，只能作为一个综合指标</t>
         </is>
@@ -1094,60 +1135,65 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>Ben、Brandon、Zane、Cory、Zander、Nancy（均为学龄期）</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Joint attention</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>joint attention was defined as shifting gaze between an object/event and another person within 5s of providing the discriminative object/event by a clinician.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>PDF第4页</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>共同注意（在物体与他人之间转换目光）</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>9个试次中的正确百分比</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>临床人员（成人）</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>自发</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>是（图1）</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>有（人物或情境，各3名被试）</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1168,60 +1214,65 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>Ben、Brandon、Zane、Cory、Zander、Nancy（均为学龄期）</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Social engagement</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Social engagement was defined as any self-initiated, independent motor or vocal behavior directed toward another to begin social interaction such as asking for help or taking the adult by the hand.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>PDF第4–5页</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>社交发起（含请求帮助、拉成人的手等）</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>9个试次中的正确百分比</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>临床人员（成人）</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>自发</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>是（图2）</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>可能（视频情境为索要玩具/食物/求助）</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="Q10" s="2" t="inlineStr">
         <is>
           <t>标签是“社交参与”，按定义实为发起，三级按定义编码</t>
         </is>
@@ -1246,60 +1297,65 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>Colin（学龄期）、Alden（学龄前期）</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>Scripted verbalizations</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Scripted verbalizations were defined as vocal statements that matched the statement of the video model. In addition, statements that were similar to the modeled response but not identical also were scored.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>PDF第5页</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>剧本式假装游戏言语（对同伴）</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>每4分钟次数（满分14–17）</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>典型发展同伴</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>剧本</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>是（图1–2）</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>有（约1个月后随访）</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>是（剧本化游戏言语）</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>只提取孤独症儿童Colin、Alden的数据，同伴Helen、Gerry是典型发展儿童，排除</t>
         </is>
@@ -1324,60 +1380,65 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>Colin（学龄期）、Alden（学龄前期）</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>Scripted play actions</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Scripted actions were defined as motor responses that matched the actions of the video model and resulted in the same change in the environment as seen in the model.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>PDF第5页</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>剧本式假装游戏动作</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>每4分钟次数（满分14–17）</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>典型发展同伴</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>剧本</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>是（图1–2）</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>是（纯游戏动作）</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1398,60 +1459,65 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>Colin（学龄期）、Alden（学龄前期）</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Unscripted verbalizations / unscripted play actions / cooperative play / reciprocal verbal interaction chains</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Cooperative play was defined as the child being within 0.33 m of the peer and engaged in the same activity ... The chain was defined as a sequence of two or more verbalizations between a participant and peer.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>PDF第5–6页</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>（不提取）</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>典型发展同伴</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>自发</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>否：原文注明data not shown或只报告均值，且只测了2次基线和2次掌握探测</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="P13" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="Q13" s="2" t="inlineStr">
         <is>
           <t>最能体现社会沟通的指标（互惠言语链）恰恰无法提取，影响本研究的归类</t>
         </is>
@@ -1468,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1477,10 +1543,11 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="27.9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10.8" customWidth="1" min="9" max="9"/>
-    <col width="31.5" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="27.9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10.8" customWidth="1" min="10" max="10"/>
+    <col width="31.5" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1506,30 +1573,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>年龄段</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>性别</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>诊断（原文）</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>诊断依据</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>按暂定规则是否纳入</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>出处</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1556,30 +1628,35 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>NSAC标准及DSM-III</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>PDF第2页</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>高功能；心理年龄3岁10个月</t>
         </is>
@@ -1606,30 +1683,35 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>PDF第2页</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1652,30 +1734,35 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>PDF第2页</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1698,30 +1785,35 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>学龄前期</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>由研究外的专业人员诊断</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1744,30 +1836,35 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>学龄前期</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>女</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1790,30 +1887,35 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>女</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1836,30 +1938,35 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1882,30 +1989,35 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>学龄前期</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>女（据原文代词）</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>PDD-NOS</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>学校心理学家评估；CARS 36（中度）；ADOS在孤独症范围</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>PDF第3–4页（表1）</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>PDD-NOS属于DSM-5孤独症谱系</t>
         </is>
@@ -1932,30 +2044,35 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>学龄前期</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>男（据原文代词）</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>PDD-NOS</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>CARS 39（重度）</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>PDF第4页（表1）</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1978,30 +2095,35 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>学龄前期</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>男（据原文代词）</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>PDD-NOS</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>CARS 37.5（重度）</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>PDF第4页（表1）</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>图1显示无明显变化</t>
         </is>
@@ -2028,30 +2150,35 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>学龄前期</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>女（据原文代词）</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>PDD-NOS</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>CARS分数原文表1未完整提取，需看原表</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>是（待核）</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>PDF第4页（表1）</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2074,30 +2201,35 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>ASD</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>医疗记录确认</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>共病ADHD、ODD</t>
         </is>
@@ -2124,30 +2256,35 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>ASD</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>医疗记录确认</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>共病ADHD</t>
         </is>
@@ -2174,30 +2311,35 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>ASD</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>医疗记录确认</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -2220,30 +2362,35 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>ASD</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>医疗记录确认</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>共病ADHD</t>
         </is>
@@ -2270,30 +2417,35 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>ASD</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>医疗记录确认</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -2316,30 +2468,35 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>女</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>ASD（学校资格类别）</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>仅学校记录中的特殊教育资格类别</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>是，但列入敏感性分析</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>诊断依据较弱；但方法部分另称所有被试经医疗记录确认，存在矛盾，需你判断</t>
         </is>
@@ -2366,30 +2523,35 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
+          <t>学龄期</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>原文只写有诊断</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2412,30 +2574,35 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
+          <t>学龄前期</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
           <t>男</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>autism</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>原文只写有诊断</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2592,10 +2759,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="54.9" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2643,6 +2810,20 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>年龄段：按被试划分、按干预开始时周岁计算；学龄前期＝3–5周岁（含5岁11个月），学龄期＝6–12周岁。同一研究的被试可分属不同年龄段。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>粒度：同一研究中不同被试的目标行为不同时，按行为分行（如Jones 2014分3行）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>页码为PDF文件页码，不是期刊页码。</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Record raw participant ages only; drop age-group and inclusion columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFWgZDD2Xx2FsxNt9VUonS
</commit_message>
<xml_diff>
--- a/编码/三级编码_试点5篇.xlsx
+++ b/编码/三级编码_试点5篇.xlsx
@@ -437,7 +437,7 @@
     <col width="25.2" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="36.9" customWidth="1" min="5" max="5"/>
+    <col width="53.1" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -475,7 +475,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>涉及被试（年龄段）</t>
+          <t>涉及被试（年龄）</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Child 1、2、3（均为学龄期）</t>
+          <t>Child 1（7岁6个月）、Child 2（6岁10个月）、Child 3（7岁10个月）</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Child 1、2、3（均为学龄期）</t>
+          <t>Child 1（7岁6个月）、Child 2（6岁10个月）、Child 3（7岁10个月）</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Child 1、2、3（均为学龄期）</t>
+          <t>Child 1（7岁6个月）、Child 2（6岁10个月）、Child 3（7岁10个月）</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>John（学龄前期）</t>
+          <t>John（4岁）</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Emma（学龄前期）、Mike（学龄期）</t>
+          <t>Emma（4岁）、Mike（6岁）</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Staci（学龄期）</t>
+          <t>Staci（6岁）</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Lucy、Tim、John、Helen（均为学龄前期）</t>
+          <t>Lucy（4岁2个月）、Tim（4岁2个月）、John（3岁10个月）、Helen（4岁2个月）</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Ben、Brandon、Zane、Cory、Zander、Nancy（均为学龄期）</t>
+          <t>Ben（8岁）、Brandon（8岁）、Zane（9岁）、Cory（11岁）、Zander（7岁）、Nancy（7岁）</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ben、Brandon、Zane、Cory、Zander、Nancy（均为学龄期）</t>
+          <t>Ben（8岁）、Brandon（8岁）、Zane（9岁）、Cory（11岁）、Zander（7岁）、Nancy（7岁）</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Colin（学龄期）、Alden（学龄前期）</t>
+          <t>Colin（7岁）、Alden（5岁）</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Colin（学龄期）、Alden（学龄前期）</t>
+          <t>Colin（7岁）、Alden（5岁）</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Colin（学龄期）、Alden（学龄前期）</t>
+          <t>Colin（7岁）、Alden（5岁）</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1534,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1543,11 +1543,9 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="27.9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10.8" customWidth="1" min="10" max="10"/>
-    <col width="31.5" customWidth="1" min="11" max="11"/>
+    <col width="27.9" customWidth="1" min="7" max="7"/>
+    <col width="10.8" customWidth="1" min="8" max="8"/>
+    <col width="40.5" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1573,35 +1571,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>年龄段</t>
+          <t>性别</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>性别</t>
+          <t>诊断（原文）</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>诊断（原文）</t>
+          <t>诊断依据</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>诊断依据</t>
+          <t>出处</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>按暂定规则是否纳入</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>出处</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1628,35 +1616,25 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>NSAC标准及DSM-III</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>NSAC标准及DSM-III</t>
+          <t>PDF第2页</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>PDF第2页</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>高功能；心理年龄3岁10个月</t>
         </is>
@@ -1683,35 +1661,25 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
           <t>PDF第2页</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1734,35 +1702,25 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
           <t>PDF第2页</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1785,35 +1743,25 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>学龄前期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>由研究外的专业人员诊断</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>由研究外的专业人员诊断</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1836,35 +1784,25 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>学龄前期</t>
+          <t>女</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1887,35 +1825,25 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>女</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1938,35 +1866,25 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>同上</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1989,35 +1907,25 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>学龄前期</t>
+          <t>女（据原文代词）</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>女（据原文代词）</t>
+          <t>PDD-NOS</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>PDD-NOS</t>
+          <t>学校心理学家评估；CARS 36（中度）；ADOS在孤独症范围</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>学校心理学家评估；CARS 36（中度）；ADOS在孤独症范围</t>
+          <t>PDF第3–4页（表1）</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>PDF第3–4页（表1）</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>PDD-NOS属于DSM-5孤独症谱系</t>
         </is>
@@ -2044,35 +1952,25 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>学龄前期</t>
+          <t>男（据原文代词）</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>男（据原文代词）</t>
+          <t>PDD-NOS</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>PDD-NOS</t>
+          <t>CARS 39（重度）</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>CARS 39（重度）</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
           <t>PDF第4页（表1）</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2095,35 +1993,25 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>学龄前期</t>
+          <t>男（据原文代词）</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>男（据原文代词）</t>
+          <t>PDD-NOS</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>PDD-NOS</t>
+          <t>CARS 37.5（重度）</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>CARS 37.5（重度）</t>
+          <t>PDF第4页（表1）</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>PDF第4页（表1）</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>图1显示无明显变化</t>
         </is>
@@ -2150,35 +2038,25 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>学龄前期</t>
+          <t>女（据原文代词）</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>女（据原文代词）</t>
+          <t>PDD-NOS</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>PDD-NOS</t>
+          <t>CARS分数原文表1未完整提取，需看原表</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>CARS分数原文表1未完整提取，需看原表</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>是（待核）</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
           <t>PDF第4页（表1）</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2201,35 +2079,25 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>ASD</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>ASD</t>
+          <t>医疗记录确认</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>医疗记录确认</t>
+          <t>PDF第3页</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>PDF第3页</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>共病ADHD、ODD</t>
         </is>
@@ -2256,35 +2124,25 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>ASD</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>ASD</t>
+          <t>医疗记录确认</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>医疗记录确认</t>
+          <t>PDF第3页</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>PDF第3页</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>共病ADHD</t>
         </is>
@@ -2311,35 +2169,25 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>ASD</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>ASD</t>
+          <t>医疗记录确认</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>医疗记录确认</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -2362,35 +2210,25 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>ASD</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>ASD</t>
+          <t>医疗记录确认</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>医疗记录确认</t>
+          <t>PDF第3页</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>PDF第3页</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>共病ADHD</t>
         </is>
@@ -2417,35 +2255,25 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>ASD</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ASD</t>
+          <t>医疗记录确认</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>医疗记录确认</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -2468,37 +2296,27 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>女</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>ASD（学校资格类别）</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ASD（学校资格类别）</t>
+          <t>仅学校记录中的特殊教育资格类别</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>仅学校记录中的特殊教育资格类别</t>
+          <t>PDF第3页</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>是，但列入敏感性分析</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>PDF第3页</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>诊断依据较弱；但方法部分另称所有被试经医疗记录确认，存在矛盾，需你判断</t>
+          <t>个人介绍中只写学校记录的资格类别；方法部分称所有被试的诊断均经医疗记录确认，两处说法不一致</t>
         </is>
       </c>
     </row>
@@ -2523,35 +2341,25 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>学龄期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>原文只写有诊断</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>原文只写有诊断</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2574,35 +2382,25 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>学龄前期</t>
+          <t>男</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>autism</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>autism</t>
+          <t>原文只写有诊断</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>原文只写有诊断</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
           <t>PDF第3页</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2759,7 +2557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2775,7 +2573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>提取范围：只提取纳入研究中、合格被试（3–12周岁、孤独症诊断）身上、有逐次数据画图的社会沟通类因变量。</t>
+          <t>提取范围：只提取纳入研究中孤独症儿童身上、有逐次数据画图的社会沟通类因变量。被试信息只记录原文事实（具体年龄、性别、诊断、诊断依据），不做分组，也不做纳入判断。</t>
         </is>
       </c>
     </row>
@@ -2803,26 +2601,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>暂定被试规则：年龄按干预开始时满3周岁、未满13周岁；诊断为明确诊断或评估工具达临界，诊断依据较弱者保留但列入敏感性分析。</t>
+          <t>粒度：同一研究中不同被试的目标行为不同时，按行为分行（如Jones 2014分3行）。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>年龄段：按被试划分、按干预开始时周岁计算；学龄前期＝3–5周岁（含5岁11个月），学龄期＝6–12周岁。同一研究的被试可分属不同年龄段。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>粒度：同一研究中不同被试的目标行为不同时，按行为分行（如Jones 2014分3行）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>页码为PDF文件页码，不是期刊页码。</t>
         </is>

</xml_diff>